<commit_message>
Add NFC column to template, NFC visibility toggle, and layout fixes
- design.xlsx now defines an NFC box-field column (was missing
  entirely, so no date could ever show NFC regardless of permissions);
  patched all existing dates' fields_enabled to match.
- Add a "Show NFC column" toggle to the Colors panel (default on),
  same show-default/per-date-override cascade as every other Colors
  setting.
- NFC column is fixed-width instead of competing equally with Model/
  CKT for flex space, and no longer renders an empty pill when a box
  has no NFC value.
- Give Splay/CKT more room now that NFC no longer crowds them.
- Fix long checkbox/radio labels in the settings panels dropping to
  their own misaligned line instead of wrapping inline with the
  input -- shared swatchLabel() helper + flex-basis:0 fix, applied
  everywhere this row pattern is used.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/design.xlsx
+++ b/design.xlsx
@@ -66,7 +66,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -171,11 +171,104 @@
         <color rgb="FF000000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -208,6 +301,21 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -573,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O25"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="2" max="2"/>
@@ -583,146 +691,120 @@
     <col width="8.619999999999999" customWidth="1" min="6" max="6"/>
     <col width="7.93" customWidth="1" min="7" max="7"/>
     <col width="4.87" customWidth="1" min="8" max="8"/>
-    <col width="4.25" customWidth="1" min="9" max="9"/>
+    <col width="4.87" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="18" t="inlineStr">
         <is>
           <t>PAGE_TITLE</t>
         </is>
       </c>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
-      <c r="M1" s="3" t="n"/>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="C1" s="19" t="n"/>
+      <c r="D1" s="19" t="n"/>
+      <c r="E1" s="19" t="n"/>
+      <c r="F1" s="19" t="n"/>
+      <c r="G1" s="19" t="n"/>
+      <c r="H1" s="19" t="n"/>
+      <c r="I1" s="19" t="n"/>
+      <c r="J1" s="19" t="n"/>
+      <c r="K1" s="19" t="n"/>
+      <c r="L1" s="19" t="n"/>
+      <c r="M1" s="19" t="n"/>
+      <c r="N1" s="20" t="n"/>
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>Venue</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>PAGE_VENUE</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="5" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="6" t="n"/>
-      <c r="G2" s="6" t="n"/>
-      <c r="H2" s="6" t="n"/>
-      <c r="I2" s="6" t="n"/>
-      <c r="J2" s="6" t="n"/>
-      <c r="K2" s="6" t="n"/>
-      <c r="L2" s="6" t="n"/>
-      <c r="M2" s="7" t="n"/>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="B2" s="21" t="n"/>
+      <c r="N2" s="22" t="n"/>
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>PAGE_DATE</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
-      <c r="J3" s="6" t="n"/>
-      <c r="K3" s="6" t="n"/>
-      <c r="L3" s="6" t="n"/>
-      <c r="M3" s="7" t="n"/>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="B3" s="21" t="n"/>
+      <c r="N3" s="22" t="n"/>
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>three</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>PAGE_THREE</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="n"/>
-      <c r="K4" s="6" t="n"/>
-      <c r="L4" s="6" t="n"/>
-      <c r="M4" s="7" t="n"/>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="B4" s="21" t="n"/>
+      <c r="N4" s="22" t="n"/>
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>four</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>PAGE_FOUR</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="9" t="n"/>
-      <c r="I5" s="9" t="n"/>
-      <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="n"/>
-      <c r="L5" s="9" t="n"/>
-      <c r="M5" s="10" t="n"/>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="B5" s="23" t="n"/>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="24" t="n"/>
+      <c r="H5" s="24" t="n"/>
+      <c r="I5" s="24" t="n"/>
+      <c r="J5" s="24" t="n"/>
+      <c r="K5" s="24" t="n"/>
+      <c r="L5" s="24" t="n"/>
+      <c r="M5" s="24" t="n"/>
+      <c r="N5" s="25" t="n"/>
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>five</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>PAGE_FIVE</t>
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="26" t="inlineStr">
         <is>
           <t>SEC1_TITLE</t>
         </is>
       </c>
-      <c r="E7" s="12" t="n"/>
-      <c r="F7" s="12" t="n"/>
-      <c r="G7" s="12" t="n"/>
-      <c r="H7" s="12" t="n"/>
-      <c r="I7" s="12" t="n"/>
-      <c r="J7" s="13" t="n"/>
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="27" t="n"/>
+      <c r="H7" s="27" t="n"/>
+      <c r="I7" s="27" t="n"/>
+      <c r="J7" s="27" t="n"/>
+      <c r="K7" s="28" t="n"/>
     </row>
     <row r="8">
       <c r="D8" s="14" t="inlineStr">
@@ -750,7 +832,12 @@
           <t>CKT</t>
         </is>
       </c>
-      <c r="J8" s="15" t="inlineStr">
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>NFC</t>
+        </is>
+      </c>
+      <c r="K8" s="15" t="inlineStr">
         <is>
           <t>Aim</t>
         </is>
@@ -778,7 +865,11 @@
         <f>CONCATENATE($D9,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J9" s="17" t="inlineStr">
+      <c r="I9" s="16">
+        <f>CONCATENATE($D9,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K9" s="17" t="inlineStr">
         <is>
           <t>SEC1_AIM</t>
         </is>
@@ -806,7 +897,11 @@
         <f>CONCATENATE($D10,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J10" s="15" t="inlineStr">
+      <c r="I10" s="16">
+        <f>CONCATENATE($D10,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K10" s="15" t="inlineStr">
         <is>
           <t>Slider</t>
         </is>
@@ -834,7 +929,11 @@
         <f>CONCATENATE($D11,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="I11" s="16">
+        <f>CONCATENATE($D11,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K11" s="17" t="inlineStr">
         <is>
           <t>SEC1_SLIDER</t>
         </is>
@@ -862,7 +961,11 @@
         <f>CONCATENATE($D12,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J12" s="15" t="inlineStr">
+      <c r="I12" s="16">
+        <f>CONCATENATE($D12,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K12" s="15" t="inlineStr">
         <is>
           <t>Total Weight</t>
         </is>
@@ -890,7 +993,11 @@
         <f>CONCATENATE($D13,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="I13" s="16">
+        <f>CONCATENATE($D13,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K13" s="17" t="inlineStr">
         <is>
           <t>SEC1_TOTALWEIGHT</t>
         </is>
@@ -918,7 +1025,11 @@
         <f>CONCATENATE($D14,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J14" s="15" t="inlineStr">
+      <c r="I14" s="16">
+        <f>CONCATENATE($D14,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K14" s="15" t="inlineStr">
         <is>
           <t>Trim (T)</t>
         </is>
@@ -946,7 +1057,11 @@
         <f>CONCATENATE($D15,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="I15" s="16">
+        <f>CONCATENATE($D15,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K15" s="17" t="inlineStr">
         <is>
           <t>SEC1_TRIMTOP</t>
         </is>
@@ -974,7 +1089,11 @@
         <f>CONCATENATE($D16,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J16" s="15" t="inlineStr">
+      <c r="I16" s="16">
+        <f>CONCATENATE($D16,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K16" s="15" t="inlineStr">
         <is>
           <t>Angle (T)</t>
         </is>
@@ -1002,7 +1121,11 @@
         <f>CONCATENATE($D17,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="I17" s="16">
+        <f>CONCATENATE($D17,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K17" s="17" t="inlineStr">
         <is>
           <t>SEC1_ANGLETOP</t>
         </is>
@@ -1030,7 +1153,11 @@
         <f>CONCATENATE($D18,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J18" s="15" t="inlineStr">
+      <c r="I18" s="16">
+        <f>CONCATENATE($D18,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K18" s="15" t="inlineStr">
         <is>
           <t>Trim (B)</t>
         </is>
@@ -1058,7 +1185,11 @@
         <f>CONCATENATE($D19,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J19" s="17" t="inlineStr">
+      <c r="I19" s="16">
+        <f>CONCATENATE($D19,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K19" s="17" t="inlineStr">
         <is>
           <t>SEC1_TRIMBOTTOM</t>
         </is>
@@ -1086,7 +1217,11 @@
         <f>CONCATENATE($D20,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J20" s="15" t="inlineStr">
+      <c r="I20" s="16">
+        <f>CONCATENATE($D20,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K20" s="15" t="inlineStr">
         <is>
           <t>Angle (B)</t>
         </is>
@@ -1114,7 +1249,11 @@
         <f>CONCATENATE($D21,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J21" s="17" t="inlineStr">
+      <c r="I21" s="16">
+        <f>CONCATENATE($D21,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
         <is>
           <t>SEC1_ANGLEBOTTOM</t>
         </is>
@@ -1142,7 +1281,11 @@
         <f>CONCATENATE($D22,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J22" s="15" t="inlineStr">
+      <c r="I22" s="16">
+        <f>CONCATENATE($D22,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K22" s="15" t="inlineStr">
         <is>
           <t>Pick (F)</t>
         </is>
@@ -1170,7 +1313,11 @@
         <f>CONCATENATE($D23,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J23" s="17" t="inlineStr">
+      <c r="I23" s="16">
+        <f>CONCATENATE($D23,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
         <is>
           <t>SEC1_PICKFRONT</t>
         </is>
@@ -1198,14 +1345,18 @@
         <f>CONCATENATE($D24,"_CIRCUIT")</f>
         <v/>
       </c>
-      <c r="J24" s="15" t="inlineStr">
+      <c r="I24" s="16">
+        <f>CONCATENATE($D24,"_NFC")</f>
+        <v/>
+      </c>
+      <c r="K24" s="15" t="inlineStr">
         <is>
           <t>Pick (R)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="J25" s="17" t="inlineStr">
+      <c r="K25" s="17" t="inlineStr">
         <is>
           <t>SEC1_PICKREAR</t>
         </is>
@@ -1213,8 +1364,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B1:M5"/>
-    <mergeCell ref="D7:J7"/>
+    <mergeCell ref="B1:N5"/>
+    <mergeCell ref="D7:K7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>